<commit_message>
finance: Bills.xlsx header row readable in Zoho; zoho:workdrive:upload --replace overwrites in place
Google's export pins every row to 15.75pt via sheet-level customHeight, so the wrapped
row-1 headers were clipped in WorkDrive/Zoho Sheet. Drop the flag on all sheets, set
row 1 to 31.5pt where headers wrap, and re-upload over the same WorkDrive file (v2.0).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance-tools/exports/bills-zoho-ready.xlsx
+++ b/finance-tools/exports/bills-zoho-ready.xlsx
@@ -674,7 +674,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AN1038"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col width="23.13" customWidth="1" style="115" min="1" max="1"/>
     <col width="14.88" customWidth="1" style="115" min="2" max="2"/>
@@ -694,7 +694,7 @@
     <col width="35.88" customWidth="1" style="115" min="22" max="22"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="31.5" customHeight="1">
       <c r="A1" s="41" t="inlineStr">
         <is>
           <t>Name</t>
@@ -18266,7 +18266,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K1002"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col width="14.13" customWidth="1" style="115" min="3" max="3"/>
     <col width="13.75" customWidth="1" style="115" min="5" max="5"/>
@@ -22889,7 +22889,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B27"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col width="25.5" customWidth="1" style="115" min="1" max="1"/>
   </cols>
@@ -23175,7 +23175,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col width="41.75" customWidth="1" style="115" min="1" max="1"/>
     <col width="8.75" customWidth="1" style="115" min="2" max="2"/>
@@ -23271,7 +23271,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AG1029"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col width="23.63" customWidth="1" style="115" min="1" max="1"/>
     <col width="21.25" customWidth="1" style="115" min="2" max="2"/>
@@ -33855,7 +33855,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q1000"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col width="14.88" customWidth="1" style="115" min="1" max="1"/>
     <col width="13.88" customWidth="1" style="115" min="2" max="2"/>
@@ -33863,7 +33863,7 @@
     <col width="11.25" customWidth="1" style="115" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="31.5" customHeight="1">
       <c r="A1" s="81" t="inlineStr">
         <is>
           <t>Accounts</t>
@@ -38962,7 +38962,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col width="9.380000000000001" customWidth="1" style="115" min="2" max="2"/>
   </cols>
@@ -43188,7 +43188,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q7"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="81" t="inlineStr">
@@ -43498,7 +43498,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col width="41.38" customWidth="1" style="115" min="1" max="1"/>
   </cols>

</xml_diff>